<commit_message>
Add Christmas Organiser listing photos and copy; align cell text vertically
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XAZTcsRbYDYsZphEU6c43B
</commit_message>
<xml_diff>
--- a/etsy-templates/Ultimate-Christmas-Organiser.xlsx
+++ b/etsy-templates/Ultimate-Christmas-Organiser.xlsx
@@ -648,10 +648,10 @@
     <t xml:space="preserve">Shuffle number</t>
   </si>
   <si>
+    <t xml:space="preserve">You're buying for</t>
+  </si>
+  <si>
     <t xml:space="preserve">Change the shuffle number for a new draw (any whole number).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">You're buying for</t>
   </si>
   <si>
     <t xml:space="preserve">Their wishlist</t>
@@ -1134,8 +1134,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1162,8 +1162,8 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1182,28 +1182,28 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="168" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1234,8 +1234,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="170" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1707,11 +1707,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="13904157"/>
-        <c:axId val="77013657"/>
+        <c:axId val="29657643"/>
+        <c:axId val="7802286"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="13904157"/>
+        <c:axId val="29657643"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1743,7 +1743,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77013657"/>
+        <c:crossAx val="7802286"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1751,7 +1751,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77013657"/>
+        <c:axId val="7802286"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1783,7 +1783,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13904157"/>
+        <c:crossAx val="29657643"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2249,11 +2249,8 @@
       <c r="C7" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="F7" s="19" t="s">
         <v>205</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>206</v>
       </c>
       <c r="G7" s="34" t="str">
         <f aca="false">IF(G6="","",IFERROR(INDEX($J$12:$J$41,MATCH(G6,$B$12:$B$41,0)),"Name not found"))</f>
@@ -2261,6 +2258,9 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="11" t="s">
+        <v>206</v>
+      </c>
       <c r="F8" s="19" t="s">
         <v>207</v>
       </c>
@@ -4688,7 +4688,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D067C166-72A1-4EEB-B3F5-4ED762345F68}</x14:id>
+          <x14:id>{B267A481-F692-4878-AEED-69C8965B3C86}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4702,7 +4702,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8F284C39-6267-4A1F-94A5-D5CC153EE454}</x14:id>
+          <x14:id>{8C6B5C3D-2B18-4040-8240-7774869CCF50}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4718,7 +4718,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D067C166-72A1-4EEB-B3F5-4ED762345F68}">
+          <x14:cfRule type="dataBar" id="{B267A481-F692-4878-AEED-69C8965B3C86}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -4733,7 +4733,7 @@
           <xm:sqref>C15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8F284C39-6267-4A1F-94A5-D5CC153EE454}">
+          <x14:cfRule type="dataBar" id="{8C6B5C3D-2B18-4040-8240-7774869CCF50}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>